<commit_message>
Match L-ka calculator to salon Raschet_L-ka layout.
Keep three material blocks, mm inputs, shared price sheet, labeled delivery and hinge holes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/prototypes/nova-2.0/Nova_2.0_салон.xlsx
+++ b/prototypes/nova-2.0/Nova_2.0_салон.xlsx
@@ -12,12 +12,13 @@
     <sheet name="Заявки_Васильево" sheetId="7" r:id="rId7"/>
     <sheet name="Продажи" sheetId="8" r:id="rId8"/>
     <sheet name="Заказы" sheetId="9" r:id="rId9"/>
-    <sheet name="Калькулятор" sheetId="10" r:id="rId10"/>
-    <sheet name="Задачи" sheetId="11" r:id="rId11"/>
-    <sheet name="Касса" sheetId="12" r:id="rId12"/>
-    <sheet name="Грузчики" sheetId="13" r:id="rId13"/>
-    <sheet name="Шпаргалки" sheetId="14" r:id="rId14"/>
-    <sheet name="Аналитика" sheetId="15" r:id="rId15"/>
+    <sheet name="Цены_Лки" sheetId="10" r:id="rId10"/>
+    <sheet name="Калькулятор" sheetId="11" r:id="rId11"/>
+    <sheet name="Задачи" sheetId="12" r:id="rId12"/>
+    <sheet name="Касса" sheetId="13" r:id="rId13"/>
+    <sheet name="Грузчики" sheetId="14" r:id="rId14"/>
+    <sheet name="Шпаргалки" sheetId="15" r:id="rId15"/>
+    <sheet name="Аналитика" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -535,170 +536,1337 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:C7"/>
   <cols>
-    <col min="1" max="1" width="40.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Калькулятор Л-ки (одна панель). Полный раскрой многих деталей — в приложении, здесь быстрый счёт.</v>
+        <v>Параметр</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Значение</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Комментарий</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>ЛДСП, ₽ за м²</v>
+      </c>
+      <c r="B2">
+        <v>1400</v>
+      </c>
+      <c r="C2" t="str">
+        <v>как в 19_08_Raschet_L-ka</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Ширина, мм</v>
+        <v>ДВП, ₽ за м²</v>
       </c>
       <c r="B3">
-        <v>2800</v>
+        <v>400</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Высота, мм</v>
+        <v>Кромка, ₽ за пог.м</v>
       </c>
       <c r="B4">
-        <v>600</v>
+        <v>250</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Материал</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Дуб Сонома</v>
+        <v>Запас ДВП</v>
+      </c>
+      <c r="B5">
+        <v>1.1</v>
+      </c>
+      <c r="C5" t="str">
+        <v>+10%, как в твоей таблице</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Кромка</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Обе стороны</v>
+        <v>Отверстие под петлю, ₽</v>
+      </c>
+      <c r="B6">
+        <v>50</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Петель, шт</v>
+        <v>Доставка, ₽</v>
       </c>
       <c r="B7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Цена м² ЛДСП</v>
-      </c>
-      <c r="B8">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Кромка: обе стороны / одна / нет</v>
-      </c>
-      <c r="B9" t="str">
-        <v>300 / 150 / 0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Петля, ₽</v>
-      </c>
-      <c r="B10">
         <v>200</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Площадь, м²</v>
-      </c>
-      <c r="B12">
-        <f>B3*B4/1000000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>ЛДСП, ₽</v>
-      </c>
-      <c r="B13">
-        <f>B12*B8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Кромка, ₽</v>
-      </c>
-      <c r="B14">
-        <f>IF(B6="Обе стороны",300,IF(OR(B6="Без кромки",B6="нет"),0,150))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Петли, ₽</v>
-      </c>
-      <c r="B15">
-        <f>B7*B10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>ИТОГО, ₽</v>
-      </c>
-      <c r="B16">
-        <f>SUM(B13:B15)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Клиент</v>
-      </c>
-      <c r="B18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Телефон</v>
-      </c>
-      <c r="B19" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Сохранить в Заказы вручную: скопируй ИТОГО и имя клиента</v>
+      <c r="C7" t="str">
+        <v>0 если клиент забирает сам</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:S25"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="4.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="4.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Клиент</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v>Телефон</v>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v>Цвет ЛДСП</v>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v>Дата</v>
+      </c>
+      <c r="H1" t="str">
+        <v>2026-09-09</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ЛДСП</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>ДВП</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v>КРОМКА</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>№</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Длина мм</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Ширина мм</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Кол-во</v>
+      </c>
+      <c r="E3" t="str">
+        <v>м²</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>№</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Длина мм</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Ширина мм</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Кол-во</v>
+      </c>
+      <c r="L3" t="str">
+        <v>м²</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v>№</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Длина мм</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Кол-во</v>
+      </c>
+      <c r="R3" t="str">
+        <v>пог.м</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4">
+        <f>IF(OR(B4="",C4="",D4=""),"",B4*C4*D4/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4">
+        <f>IF(OR(I4="",J4="",K4=""),"",I4*J4*K4/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4">
+        <f>IF(OR(P4="",Q4=""),"",P4*Q4/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5">
+        <f>IF(OR(B5="",C5="",D5=""),"",B5*C5*D5/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5">
+        <f>IF(OR(I5="",J5="",K5=""),"",I5*J5*K5/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5">
+        <v>2</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5">
+        <f>IF(OR(P5="",Q5=""),"",P5*Q5/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6">
+        <f>IF(OR(B6="",C6="",D6=""),"",B6*C6*D6/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6">
+        <f>IF(OR(I6="",J6="",K6=""),"",I6*J6*K6/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6">
+        <v>3</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6">
+        <f>IF(OR(P6="",Q6=""),"",P6*Q6/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7">
+        <f>IF(OR(B7="",C7="",D7=""),"",B7*C7*D7/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7">
+        <v>4</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7">
+        <f>IF(OR(I7="",J7="",K7=""),"",I7*J7*K7/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7">
+        <v>4</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7">
+        <f>IF(OR(P7="",Q7=""),"",P7*Q7/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IF(OR(B8="",C8="",D8=""),"",B8*C8*D8/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8">
+        <v>5</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8">
+        <f>IF(OR(I8="",J8="",K8=""),"",I8*J8*K8/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8">
+        <v>5</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8">
+        <f>IF(OR(P8="",Q8=""),"",P8*Q8/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>6</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9">
+        <f>IF(OR(B9="",C9="",D9=""),"",B9*C9*D9/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9">
+        <v>6</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9">
+        <f>IF(OR(I9="",J9="",K9=""),"",I9*J9*K9/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9">
+        <v>6</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9">
+        <f>IF(OR(P9="",Q9=""),"",P9*Q9/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10">
+        <f>IF(OR(B10="",C10="",D10=""),"",B10*C10*D10/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10">
+        <v>7</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10">
+        <f>IF(OR(I10="",J10="",K10=""),"",I10*J10*K10/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10">
+        <v>7</v>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10">
+        <f>IF(OR(P10="",Q10=""),"",P10*Q10/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>8</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11">
+        <f>IF(OR(B11="",C11="",D11=""),"",B11*C11*D11/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11">
+        <v>8</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11">
+        <f>IF(OR(I11="",J11="",K11=""),"",I11*J11*K11/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11">
+        <v>8</v>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11">
+        <f>IF(OR(P11="",Q11=""),"",P11*Q11/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>9</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12">
+        <f>IF(OR(B12="",C12="",D12=""),"",B12*C12*D12/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12">
+        <v>9</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12">
+        <f>IF(OR(I12="",J12="",K12=""),"",I12*J12*K12/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12">
+        <v>9</v>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12">
+        <f>IF(OR(P12="",Q12=""),"",P12*Q12/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>10</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13">
+        <f>IF(OR(B13="",C13="",D13=""),"",B13*C13*D13/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13">
+        <v>10</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13">
+        <f>IF(OR(I13="",J13="",K13=""),"",I13*J13*K13/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13">
+        <v>10</v>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13">
+        <f>IF(OR(P13="",Q13=""),"",P13*Q13/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>11</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14">
+        <f>IF(OR(B14="",C14="",D14=""),"",B14*C14*D14/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14">
+        <v>11</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14">
+        <f>IF(OR(I14="",J14="",K14=""),"",I14*J14*K14/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14">
+        <v>11</v>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14">
+        <f>IF(OR(P14="",Q14=""),"",P14*Q14/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>12</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15">
+        <f>IF(OR(B15="",C15="",D15=""),"",B15*C15*D15/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15">
+        <v>12</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15">
+        <f>IF(OR(I15="",J15="",K15=""),"",I15*J15*K15/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15">
+        <v>12</v>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15">
+        <f>IF(OR(P15="",Q15=""),"",P15*Q15/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>13</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16">
+        <f>IF(OR(B16="",C16="",D16=""),"",B16*C16*D16/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16">
+        <v>13</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16">
+        <f>IF(OR(I16="",J16="",K16=""),"",I16*J16*K16/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16">
+        <v>13</v>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16">
+        <f>IF(OR(P16="",Q16=""),"",P16*Q16/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>14</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17">
+        <f>IF(OR(B17="",C17="",D17=""),"",B17*C17*D17/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17">
+        <v>14</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17">
+        <f>IF(OR(I17="",J17="",K17=""),"",I17*J17*K17/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17">
+        <v>14</v>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17">
+        <f>IF(OR(P17="",Q17=""),"",P17*Q17/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>15</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18">
+        <f>IF(OR(B18="",C18="",D18=""),"",B18*C18*D18/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18">
+        <v>15</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18">
+        <f>IF(OR(I18="",J18="",K18=""),"",I18*J18*K18/1000000)</f>
+        <v>0</v>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18">
+        <v>15</v>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18">
+        <f>IF(OR(P18="",Q18=""),"",P18*Q18/1000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>м² итого</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19">
+        <f>SUM(E4:E18)</f>
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <f>Цены_Лки!B2</f>
+        <v>0</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v>м² итого</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19">
+        <f>SUM(L4:L18)</f>
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <f>Цены_Лки!B3</f>
+        <v>0</v>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v>пог.м итого</v>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19">
+        <f>SUM(R4:R18)</f>
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <f>Цены_Лки!B4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>сумма ЛДСП</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20">
+        <f>E19*F19</f>
+        <v>0</v>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v>сумма ДВП (+10%)</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20">
+        <f>L19*Цены_Лки!B5*M19</f>
+        <v>0</v>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v>сумма кромки</v>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20">
+        <f>R19*S19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Отверстия под петли, шт</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22" t="str">
+        <v>× цена</v>
+      </c>
+      <c r="D22">
+        <f>Цены_Лки!B6</f>
+        <v>0</v>
+      </c>
+      <c r="E22" t="str">
+        <v>=</v>
+      </c>
+      <c r="F22">
+        <f>B22*D22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Доставка</v>
+      </c>
+      <c r="B23">
+        <f>Цены_Лки!B7</f>
+        <v>0</v>
+      </c>
+      <c r="C23" t="str">
+        <v/>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v>=</v>
+      </c>
+      <c r="F23">
+        <f>B23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>ИТОГО</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v>=</v>
+      </c>
+      <c r="F24">
+        <f>F20+M20+S20+F22+F23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Размеры в мм. Цены — лист Цены_Лки. Три блока как в 19_08_Raschet_L-ka.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:S25"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E10"/>
   <cols>
@@ -886,7 +2054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L2"/>
   <cols>
@@ -988,7 +2156,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G2"/>
   <cols>
@@ -1054,7 +2222,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C8"/>
   <cols>
@@ -1158,7 +2326,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
   <cols>

</xml_diff>

<commit_message>
Add click-style L-ka calculator matching the web parts list.
Use on/off and edge flags instead of typing meters; optional Apps Script menu adds parts and copies the total into Orders.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/prototypes/nova-2.0/Nova_2.0_салон.xlsx
+++ b/prototypes/nova-2.0/Nova_2.0_салон.xlsx
@@ -4,21 +4,23 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Главная" sheetId="1" r:id="rId1"/>
-    <sheet name="Калькулятор" sheetId="2" r:id="rId2"/>
-    <sheet name="Цены_Лки" sheetId="3" r:id="rId3"/>
-    <sheet name="Заказы" sheetId="4" r:id="rId4"/>
-    <sheet name="Фурнитура" sheetId="5" r:id="rId5"/>
-    <sheet name="Продажи" sheetId="6" r:id="rId6"/>
-    <sheet name="Касса" sheetId="7" r:id="rId7"/>
-    <sheet name="Задачи" sheetId="8" r:id="rId8"/>
-    <sheet name="Заявки_Рондо" sheetId="9" r:id="rId9"/>
-    <sheet name="Заявки_Партнер" sheetId="10" r:id="rId10"/>
-    <sheet name="Заявки_Васильево" sheetId="11" r:id="rId11"/>
-    <sheet name="Грузчики" sheetId="12" r:id="rId12"/>
-    <sheet name="Шпаргалки" sheetId="13" r:id="rId13"/>
-    <sheet name="Поставщики" sheetId="14" r:id="rId14"/>
-    <sheet name="Аналитика" sheetId="15" r:id="rId15"/>
-    <sheet name="Старт" sheetId="16" r:id="rId16"/>
+    <sheet name="Кальк_веб" sheetId="2" r:id="rId2"/>
+    <sheet name="Калькулятор" sheetId="3" r:id="rId3"/>
+    <sheet name="Материалы_Лки" sheetId="4" r:id="rId4"/>
+    <sheet name="Цены_Лки" sheetId="5" r:id="rId5"/>
+    <sheet name="Заказы" sheetId="6" r:id="rId6"/>
+    <sheet name="Фурнитура" sheetId="7" r:id="rId7"/>
+    <sheet name="Продажи" sheetId="8" r:id="rId8"/>
+    <sheet name="Касса" sheetId="9" r:id="rId9"/>
+    <sheet name="Задачи" sheetId="10" r:id="rId10"/>
+    <sheet name="Заявки_Рондо" sheetId="11" r:id="rId11"/>
+    <sheet name="Заявки_Партнер" sheetId="12" r:id="rId12"/>
+    <sheet name="Заявки_Васильево" sheetId="13" r:id="rId13"/>
+    <sheet name="Грузчики" sheetId="14" r:id="rId14"/>
+    <sheet name="Шпаргалки" sheetId="15" r:id="rId15"/>
+    <sheet name="Поставщики" sheetId="16" r:id="rId16"/>
+    <sheet name="Аналитика" sheetId="17" r:id="rId17"/>
+    <sheet name="Старт" sheetId="18" r:id="rId18"/>
   </sheets>
 </workbook>
 </file>
@@ -539,7 +541,7 @@
     </row>
     <row r="6">
       <c r="A6">
-        <f>HYPERLINK("#Калькулятор!A1","→ Калькулятор Л-ок")</f>
+        <f>HYPERLINK("#Кальк_веб!A1","→ Калькулятор как на сайте")</f>
         <v>0</v>
       </c>
       <c r="B6" t="str">
@@ -636,24 +638,188 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E10"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" customWidth="1"/>
+    <col min="3" max="3" width="78.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1">
-        <f>QUERY(Фурнитура!A:H;"select A,B,G,H where C = 'Партнер' and H &gt; 0";1)</f>
-        <v>0</v>
+      <c r="A1" t="str">
+        <v>Категория</v>
+      </c>
+      <c r="B1" t="str">
+        <v>№</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Действие</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Готово (да/нет)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Комментарий</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Утро</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Включить Инфопредприятие → интерфейс кассира</v>
+      </c>
+      <c r="D2" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Утро</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Пересчитать наличку и сверить с «должно быть» на листе Касса</v>
+      </c>
+      <c r="D3" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Утро</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Чеки: сумма на чеках = сумма в программе</v>
+      </c>
+      <c r="D4" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>День</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Продажи фурнитуры писать на лист Продажи (нал / карта)</v>
+      </c>
+      <c r="D5" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>День</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Новый распил — Калькулятор, потом строка на Заказы</v>
+      </c>
+      <c r="D6" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Закрытие</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Инфо: эквайринг АВТО → Д/Р</v>
+      </c>
+      <c r="D7" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Закрытие</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Инфо: поступление в кассу АВТО → Д/Р</v>
+      </c>
+      <c r="D8" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Закрытие</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Отдать проверенные чеки бухгалтеру</v>
+      </c>
+      <c r="D9" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Закрытие</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Сверить остаток в программе и факт на Фурнитуре</v>
+      </c>
+      <c r="D10" t="str">
+        <v>нет</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -671,7 +837,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>QUERY(Фурнитура!A:H;"select A,B,G,H where C = 'Васильево / Ортус' and H &gt; 0";1)</f>
+        <f>QUERY(Фурнитура!A:H;"select A,B,G,H where C = 'Рондо / Ладья' and H &gt; 0";1)</f>
         <v>0</v>
       </c>
     </row>
@@ -683,6 +849,54 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1">
+        <f>QUERY(Фурнитура!A:H;"select A,B,G,H where C = 'Партнер' and H &gt; 0";1)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1">
+        <f>QUERY(Фурнитура!A:H;"select A,B,G,H where C = 'Васильево / Ортус' and H &gt; 0";1)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G2"/>
   <cols>
@@ -748,7 +962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C8"/>
   <cols>
@@ -852,7 +1066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A4"/>
   <cols>
@@ -886,7 +1100,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
   <cols>
@@ -979,7 +1193,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A22"/>
   <cols>
@@ -1104,6 +1318,596 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N17"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ИТОГО, ₽</v>
+      </c>
+      <c r="B1">
+        <f>IF(J17="","",J17+L17+N17)</f>
+        <v>0</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Листов</v>
+      </c>
+      <c r="D1">
+        <f>H17</f>
+        <v>0</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Как в веб-калькуляторе: галочки кромок, готовые детали. В Google: колонки Вкл и 4 кромки → Данные → Флажок.</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Материал (как в списке Материалы_Лки)</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ЛДСП 16 мм Дуб Сонома</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Цена листа</v>
+      </c>
+      <c r="D2">
+        <f>IFERROR(VLOOKUP(B2,Материалы_Лки!A:E,5,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Распил ₽/пог.м</v>
+      </c>
+      <c r="F2">
+        <v>35</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Кромка ₽/пог.м</v>
+      </c>
+      <c r="H2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Клиент</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>Телефон</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>КПД раскроя</v>
+      </c>
+      <c r="F3">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Вкл</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Деталь</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Длина мм</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Ширина мм</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Шт</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Кромка длин.1</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Кромка длин.2</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Кромка шир.1</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Кромка шир.2</v>
+      </c>
+      <c r="J5" t="str">
+        <v>м²</v>
+      </c>
+      <c r="K5" t="str">
+        <v>кромка пог.м</v>
+      </c>
+      <c r="L5" t="str">
+        <v>пил пог.м</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Боковина вертикальная</v>
+      </c>
+      <c r="C6">
+        <v>2000</v>
+      </c>
+      <c r="D6">
+        <v>580</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <f>IF(A6&lt;&gt;TRUE,"",ROUND(C6*D6*E6/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <f>IF(A6&lt;&gt;TRUE,"",ROUND((N(F6)*C6+N(G6)*C6+N(H6)*D6+N(I6)*D6)*E6/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <f>IF(A6&lt;&gt;TRUE,"",ROUND((C6+D6)*2*E6/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Дно / Крыша</v>
+      </c>
+      <c r="C7">
+        <v>768</v>
+      </c>
+      <c r="D7">
+        <v>580</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <f>IF(A7&lt;&gt;TRUE,"",ROUND(C7*D7*E7/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <f>IF(A7&lt;&gt;TRUE,"",ROUND((N(F7)*C7+N(G7)*C7+N(H7)*D7+N(I7)*D7)*E7/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <f>IF(A7&lt;&gt;TRUE,"",ROUND((C7+D7)*2*E7/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Полка вкладная</v>
+      </c>
+      <c r="C8">
+        <v>768</v>
+      </c>
+      <c r="D8">
+        <v>550</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <f>IF(A8&lt;&gt;TRUE,"",ROUND(C8*D8*E8/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <f>IF(A8&lt;&gt;TRUE,"",ROUND((N(F8)*C8+N(G8)*C8+N(H8)*D8+N(I8)*D8)*E8/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <f>IF(A8&lt;&gt;TRUE,"",ROUND((C8+D8)*2*E8/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Стойка / перегородка</v>
+      </c>
+      <c r="C9">
+        <v>2000</v>
+      </c>
+      <c r="D9">
+        <v>400</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <f>IF(A9&lt;&gt;TRUE,"",ROUND(C9*D9*E9/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <f>IF(A9&lt;&gt;TRUE,"",ROUND((N(F9)*C9+N(G9)*C9+N(H9)*D9+N(I9)*D9)*E9/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <f>IF(A9&lt;&gt;TRUE,"",ROUND((C9+D9)*2*E9/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="b">
+        <v>0</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Фасад</v>
+      </c>
+      <c r="C10">
+        <v>700</v>
+      </c>
+      <c r="D10">
+        <v>400</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <f>IF(A10&lt;&gt;TRUE,"",ROUND(C10*D10*E10/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <f>IF(A10&lt;&gt;TRUE,"",ROUND((N(F10)*C10+N(G10)*C10+N(H10)*D10+N(I10)*D10)*E10/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <f>IF(A10&lt;&gt;TRUE,"",ROUND((C10+D10)*2*E10/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <f>IF(A11&lt;&gt;TRUE,"",ROUND(C11*D11*E11/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <f>IF(A11&lt;&gt;TRUE,"",ROUND((N(F11)*C11+N(G11)*C11+N(H11)*D11+N(I11)*D11)*E11/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <f>IF(A11&lt;&gt;TRUE,"",ROUND((C11+D11)*2*E11/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="b">
+        <v>0</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <f>IF(A12&lt;&gt;TRUE,"",ROUND(C12*D12*E12/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <f>IF(A12&lt;&gt;TRUE,"",ROUND((N(F12)*C12+N(G12)*C12+N(H12)*D12+N(I12)*D12)*E12/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <f>IF(A12&lt;&gt;TRUE,"",ROUND((C12+D12)*2*E12/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="b">
+        <v>0</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <f>IF(A13&lt;&gt;TRUE,"",ROUND(C13*D13*E13/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <f>IF(A13&lt;&gt;TRUE,"",ROUND((N(F13)*C13+N(G13)*C13+N(H13)*D13+N(I13)*D13)*E13/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <f>IF(A13&lt;&gt;TRUE,"",ROUND((C13+D13)*2*E13/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="b">
+        <v>0</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <f>IF(A14&lt;&gt;TRUE,"",ROUND(C14*D14*E14/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <f>IF(A14&lt;&gt;TRUE,"",ROUND((N(F14)*C14+N(G14)*C14+N(H14)*D14+N(I14)*D14)*E14/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <f>IF(A14&lt;&gt;TRUE,"",ROUND((C14+D14)*2*E14/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="b">
+        <v>0</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="b">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <f>IF(A15&lt;&gt;TRUE,"",ROUND(C15*D15*E15/1000000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <f>IF(A15&lt;&gt;TRUE,"",ROUND((N(F15)*C15+N(G15)*C15+N(H15)*D15+N(I15)*D15)*E15/1000,3))</f>
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <f>IF(A15&lt;&gt;TRUE,"",ROUND((C15+D15)*2*E15/1000,3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>м² деталей</v>
+      </c>
+      <c r="B17">
+        <f>SUM(J6:J15)</f>
+        <v>0</v>
+      </c>
+      <c r="C17" t="str">
+        <v>кромка м</v>
+      </c>
+      <c r="D17">
+        <f>SUM(K6:K15)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" t="str">
+        <v>пил м</v>
+      </c>
+      <c r="F17">
+        <f>SUM(L6:L15)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" t="str">
+        <v>листы</v>
+      </c>
+      <c r="H17">
+        <f>IF(B17=0,"",ROUNDUP(B17/(IFERROR(VLOOKUP(B2,Материалы_Лки!A:C,2,FALSE),2750)*IFERROR(VLOOKUP(B2,Материалы_Лки!A:C,3,FALSE),1830)/1000000*F3),0))</f>
+        <v>0</v>
+      </c>
+      <c r="I17" t="str">
+        <v>ЛДСП ₽</v>
+      </c>
+      <c r="J17">
+        <f>ROUND(H17*D2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K17" t="str">
+        <v>кромка ₽</v>
+      </c>
+      <c r="L17">
+        <f>ROUND(D17*H2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M17" t="str">
+        <v>распил ₽</v>
+      </c>
+      <c r="N17">
+        <f>ROUND(F17*F2*0.55,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N17"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S25"/>
   <cols>
@@ -2356,7 +3160,166 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F7"/>
+  <cols>
+    <col min="1" max="1" width="36.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Название</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Длина листа мм</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Ширина листа мм</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Толщина</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Цена листа</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Поставщик</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ЛДСП 16 мм Дуб Сонома</v>
+      </c>
+      <c r="B2">
+        <v>2750</v>
+      </c>
+      <c r="C2">
+        <v>1830</v>
+      </c>
+      <c r="D2">
+        <v>16</v>
+      </c>
+      <c r="E2">
+        <v>2450</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Партнер</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ЛДСП 16 мм Белый</v>
+      </c>
+      <c r="B3">
+        <v>2750</v>
+      </c>
+      <c r="C3">
+        <v>1830</v>
+      </c>
+      <c r="D3">
+        <v>16</v>
+      </c>
+      <c r="E3">
+        <v>2200</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Партнер</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ЛДСП 16 мм Серый Графит</v>
+      </c>
+      <c r="B4">
+        <v>2800</v>
+      </c>
+      <c r="C4">
+        <v>2070</v>
+      </c>
+      <c r="D4">
+        <v>16</v>
+      </c>
+      <c r="E4">
+        <v>2950</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Рондо / Ладья</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ЛДСП 16 мм Дуб Вотан</v>
+      </c>
+      <c r="B5">
+        <v>2750</v>
+      </c>
+      <c r="C5">
+        <v>1830</v>
+      </c>
+      <c r="D5">
+        <v>16</v>
+      </c>
+      <c r="E5">
+        <v>2600</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Рондо / Ладья</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ЛДСП 16 мм Венге</v>
+      </c>
+      <c r="B6">
+        <v>2750</v>
+      </c>
+      <c r="C6">
+        <v>1830</v>
+      </c>
+      <c r="D6">
+        <v>16</v>
+      </c>
+      <c r="E6">
+        <v>2400</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Васильево / Ортус</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ДВП 3.2 мм</v>
+      </c>
+      <c r="B7">
+        <v>2750</v>
+      </c>
+      <c r="C7">
+        <v>1700</v>
+      </c>
+      <c r="D7">
+        <v>3.2</v>
+      </c>
+      <c r="E7">
+        <v>950</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Васильево / Ортус</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C8"/>
   <cols>
@@ -2460,7 +3423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M11"/>
   <cols>
@@ -2967,7 +3930,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P16"/>
   <cols>
@@ -3824,7 +4787,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I16"/>
   <cols>
@@ -4325,7 +5288,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L2"/>
   <cols>
@@ -4425,216 +5388,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="6.83203125" customWidth="1"/>
-    <col min="3" max="3" width="78.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Категория</v>
-      </c>
-      <c r="B1" t="str">
-        <v>№</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Действие</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Готово (да/нет)</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Комментарий</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Утро</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Включить Инфопредприятие → интерфейс кассира</v>
-      </c>
-      <c r="D2" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Утро</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Пересчитать наличку и сверить с «должно быть» на листе Касса</v>
-      </c>
-      <c r="D3" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Утро</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Чеки: сумма на чеках = сумма в программе</v>
-      </c>
-      <c r="D4" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>День</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Продажи фурнитуры писать на лист Продажи (нал / карта)</v>
-      </c>
-      <c r="D5" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>День</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Новый распил — Калькулятор, потом строка на Заказы</v>
-      </c>
-      <c r="D6" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Закрытие</v>
-      </c>
-      <c r="B7">
-        <v>6</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Инфо: эквайринг АВТО → Д/Р</v>
-      </c>
-      <c r="D7" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Закрытие</v>
-      </c>
-      <c r="B8">
-        <v>7</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Инфо: поступление в кассу АВТО → Д/Р</v>
-      </c>
-      <c r="D8" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Закрытие</v>
-      </c>
-      <c r="B9">
-        <v>8</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Отдать проверенные чеки бухгалтеру</v>
-      </c>
-      <c r="D9" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Закрытие</v>
-      </c>
-      <c r="B10">
-        <v>9</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Сверить остаток в программе и факт на Фурнитуре</v>
-      </c>
-      <c r="D10" t="str">
-        <v>нет</v>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1">
-        <f>QUERY(Фурнитура!A:H;"select A,B,G,H where C = 'Рондо / Ладья' and H &gt; 0";1)</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Russian locale flags in the web-style calculator.
Use 1/0 instead of TRUE/FALSE so Excel does not show ИСТИНА/ЛОЖЬ, and accept да/ИСТИНА if a sheet already has those words.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/prototypes/nova-2.0/Nova_2.0_салон.xlsx
+++ b/prototypes/nova-2.0/Nova_2.0_салон.xlsx
@@ -1351,7 +1351,7 @@
         <v>0</v>
       </c>
       <c r="E1" t="str">
-        <v>Как в веб-калькуляторе: галочки кромок, готовые детали. В Google: колонки Вкл и 4 кромки → Данные → Флажок.</v>
+        <v>Вкл и кромки: ставь 1 или 0 (не ИСТИНА). В Google потом можно Вставка → Флажок — формулы всё равно сработают.</v>
       </c>
     </row>
     <row r="2">
@@ -1403,7 +1403,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Вкл</v>
+        <v>Вкл 1=да</v>
       </c>
       <c r="B5" t="str">
         <v>Деталь</v>
@@ -1440,7 +1440,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="b">
+      <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" t="str">
@@ -1455,33 +1455,33 @@
       <c r="E6">
         <v>2</v>
       </c>
-      <c r="F6" t="b">
+      <c r="F6">
         <v>1</v>
       </c>
-      <c r="G6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H6" t="b">
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>1</v>
       </c>
-      <c r="I6" t="b">
+      <c r="I6">
         <v>1</v>
       </c>
       <c r="J6">
-        <f>IF(A6&lt;&gt;TRUE,"",ROUND(C6*D6*E6/1000000,3))</f>
+        <f>IF(OR(A6=1,A6="да",A6="ДА",A6="ИСТИНА"),ROUND(C6*D6*E6/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K6">
-        <f>IF(A6&lt;&gt;TRUE,"",ROUND((N(F6)*C6+N(G6)*C6+N(H6)*D6+N(I6)*D6)*E6/1000,3))</f>
+        <f>IF(OR(A6=1,A6="да",A6="ДА",A6="ИСТИНА"),ROUND((IF(OR(F6=1,F6="да",F6="ДА",F6="ИСТИНА"),C6,0)+IF(OR(G6=1,G6="да",G6="ДА",G6="ИСТИНА"),C6,0)+IF(OR(H6=1,H6="да",H6="ДА",H6="ИСТИНА"),D6,0)+IF(OR(I6=1,I6="да",I6="ДА",I6="ИСТИНА"),D6,0))*E6/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L6">
-        <f>IF(A6&lt;&gt;TRUE,"",ROUND((C6+D6)*2*E6/1000,3))</f>
+        <f>IF(OR(A6=1,A6="да",A6="ДА",A6="ИСТИНА"),ROUND((C6+D6)*2*E6/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="b">
+      <c r="A7">
         <v>1</v>
       </c>
       <c r="B7" t="str">
@@ -1496,33 +1496,33 @@
       <c r="E7">
         <v>2</v>
       </c>
-      <c r="F7" t="b">
+      <c r="F7">
         <v>1</v>
       </c>
-      <c r="G7" t="b">
-        <v>0</v>
-      </c>
-      <c r="H7" t="b">
-        <v>0</v>
-      </c>
-      <c r="I7" t="b">
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <f>IF(A7&lt;&gt;TRUE,"",ROUND(C7*D7*E7/1000000,3))</f>
+        <f>IF(OR(A7=1,A7="да",A7="ДА",A7="ИСТИНА"),ROUND(C7*D7*E7/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K7">
-        <f>IF(A7&lt;&gt;TRUE,"",ROUND((N(F7)*C7+N(G7)*C7+N(H7)*D7+N(I7)*D7)*E7/1000,3))</f>
+        <f>IF(OR(A7=1,A7="да",A7="ДА",A7="ИСТИНА"),ROUND((IF(OR(F7=1,F7="да",F7="ДА",F7="ИСТИНА"),C7,0)+IF(OR(G7=1,G7="да",G7="ДА",G7="ИСТИНА"),C7,0)+IF(OR(H7=1,H7="да",H7="ДА",H7="ИСТИНА"),D7,0)+IF(OR(I7=1,I7="да",I7="ДА",I7="ИСТИНА"),D7,0))*E7/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L7">
-        <f>IF(A7&lt;&gt;TRUE,"",ROUND((C7+D7)*2*E7/1000,3))</f>
+        <f>IF(OR(A7=1,A7="да",A7="ДА",A7="ИСТИНА"),ROUND((C7+D7)*2*E7/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="b">
+      <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="str">
@@ -1537,33 +1537,33 @@
       <c r="E8">
         <v>3</v>
       </c>
-      <c r="F8" t="b">
+      <c r="F8">
         <v>1</v>
       </c>
-      <c r="G8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H8" t="b">
-        <v>0</v>
-      </c>
-      <c r="I8" t="b">
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <f>IF(A8&lt;&gt;TRUE,"",ROUND(C8*D8*E8/1000000,3))</f>
+        <f>IF(OR(A8=1,A8="да",A8="ДА",A8="ИСТИНА"),ROUND(C8*D8*E8/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K8">
-        <f>IF(A8&lt;&gt;TRUE,"",ROUND((N(F8)*C8+N(G8)*C8+N(H8)*D8+N(I8)*D8)*E8/1000,3))</f>
+        <f>IF(OR(A8=1,A8="да",A8="ДА",A8="ИСТИНА"),ROUND((IF(OR(F8=1,F8="да",F8="ДА",F8="ИСТИНА"),C8,0)+IF(OR(G8=1,G8="да",G8="ДА",G8="ИСТИНА"),C8,0)+IF(OR(H8=1,H8="да",H8="ДА",H8="ИСТИНА"),D8,0)+IF(OR(I8=1,I8="да",I8="ДА",I8="ИСТИНА"),D8,0))*E8/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L8">
-        <f>IF(A8&lt;&gt;TRUE,"",ROUND((C8+D8)*2*E8/1000,3))</f>
+        <f>IF(OR(A8=1,A8="да",A8="ДА",A8="ИСТИНА"),ROUND((C8+D8)*2*E8/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="b">
+      <c r="A9">
         <v>0</v>
       </c>
       <c r="B9" t="str">
@@ -1578,33 +1578,33 @@
       <c r="E9">
         <v>1</v>
       </c>
-      <c r="F9" t="b">
+      <c r="F9">
         <v>1</v>
       </c>
-      <c r="G9" t="b">
-        <v>0</v>
-      </c>
-      <c r="H9" t="b">
-        <v>0</v>
-      </c>
-      <c r="I9" t="b">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
         <v>0</v>
       </c>
       <c r="J9">
-        <f>IF(A9&lt;&gt;TRUE,"",ROUND(C9*D9*E9/1000000,3))</f>
+        <f>IF(OR(A9=1,A9="да",A9="ДА",A9="ИСТИНА"),ROUND(C9*D9*E9/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K9">
-        <f>IF(A9&lt;&gt;TRUE,"",ROUND((N(F9)*C9+N(G9)*C9+N(H9)*D9+N(I9)*D9)*E9/1000,3))</f>
+        <f>IF(OR(A9=1,A9="да",A9="ДА",A9="ИСТИНА"),ROUND((IF(OR(F9=1,F9="да",F9="ДА",F9="ИСТИНА"),C9,0)+IF(OR(G9=1,G9="да",G9="ДА",G9="ИСТИНА"),C9,0)+IF(OR(H9=1,H9="да",H9="ДА",H9="ИСТИНА"),D9,0)+IF(OR(I9=1,I9="да",I9="ДА",I9="ИСТИНА"),D9,0))*E9/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L9">
-        <f>IF(A9&lt;&gt;TRUE,"",ROUND((C9+D9)*2*E9/1000,3))</f>
+        <f>IF(OR(A9=1,A9="да",A9="ДА",A9="ИСТИНА"),ROUND((C9+D9)*2*E9/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="b">
+      <c r="A10">
         <v>0</v>
       </c>
       <c r="B10" t="str">
@@ -1619,33 +1619,33 @@
       <c r="E10">
         <v>2</v>
       </c>
-      <c r="F10" t="b">
+      <c r="F10">
         <v>1</v>
       </c>
-      <c r="G10" t="b">
+      <c r="G10">
         <v>1</v>
       </c>
-      <c r="H10" t="b">
+      <c r="H10">
         <v>1</v>
       </c>
-      <c r="I10" t="b">
+      <c r="I10">
         <v>1</v>
       </c>
       <c r="J10">
-        <f>IF(A10&lt;&gt;TRUE,"",ROUND(C10*D10*E10/1000000,3))</f>
+        <f>IF(OR(A10=1,A10="да",A10="ДА",A10="ИСТИНА"),ROUND(C10*D10*E10/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K10">
-        <f>IF(A10&lt;&gt;TRUE,"",ROUND((N(F10)*C10+N(G10)*C10+N(H10)*D10+N(I10)*D10)*E10/1000,3))</f>
+        <f>IF(OR(A10=1,A10="да",A10="ДА",A10="ИСТИНА"),ROUND((IF(OR(F10=1,F10="да",F10="ДА",F10="ИСТИНА"),C10,0)+IF(OR(G10=1,G10="да",G10="ДА",G10="ИСТИНА"),C10,0)+IF(OR(H10=1,H10="да",H10="ДА",H10="ИСТИНА"),D10,0)+IF(OR(I10=1,I10="да",I10="ДА",I10="ИСТИНА"),D10,0))*E10/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L10">
-        <f>IF(A10&lt;&gt;TRUE,"",ROUND((C10+D10)*2*E10/1000,3))</f>
+        <f>IF(OR(A10=1,A10="да",A10="ДА",A10="ИСТИНА"),ROUND((C10+D10)*2*E10/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="b">
+      <c r="A11">
         <v>0</v>
       </c>
       <c r="B11" t="str">
@@ -1660,33 +1660,33 @@
       <c r="E11" t="str">
         <v/>
       </c>
-      <c r="F11" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" t="b">
-        <v>0</v>
-      </c>
-      <c r="H11" t="b">
-        <v>0</v>
-      </c>
-      <c r="I11" t="b">
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <f>IF(A11&lt;&gt;TRUE,"",ROUND(C11*D11*E11/1000000,3))</f>
+        <f>IF(OR(A11=1,A11="да",A11="ДА",A11="ИСТИНА"),ROUND(C11*D11*E11/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K11">
-        <f>IF(A11&lt;&gt;TRUE,"",ROUND((N(F11)*C11+N(G11)*C11+N(H11)*D11+N(I11)*D11)*E11/1000,3))</f>
+        <f>IF(OR(A11=1,A11="да",A11="ДА",A11="ИСТИНА"),ROUND((IF(OR(F11=1,F11="да",F11="ДА",F11="ИСТИНА"),C11,0)+IF(OR(G11=1,G11="да",G11="ДА",G11="ИСТИНА"),C11,0)+IF(OR(H11=1,H11="да",H11="ДА",H11="ИСТИНА"),D11,0)+IF(OR(I11=1,I11="да",I11="ДА",I11="ИСТИНА"),D11,0))*E11/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L11">
-        <f>IF(A11&lt;&gt;TRUE,"",ROUND((C11+D11)*2*E11/1000,3))</f>
+        <f>IF(OR(A11=1,A11="да",A11="ДА",A11="ИСТИНА"),ROUND((C11+D11)*2*E11/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="b">
+      <c r="A12">
         <v>0</v>
       </c>
       <c r="B12" t="str">
@@ -1701,33 +1701,33 @@
       <c r="E12" t="str">
         <v/>
       </c>
-      <c r="F12" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12" t="b">
-        <v>0</v>
-      </c>
-      <c r="I12" t="b">
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
         <v>0</v>
       </c>
       <c r="J12">
-        <f>IF(A12&lt;&gt;TRUE,"",ROUND(C12*D12*E12/1000000,3))</f>
+        <f>IF(OR(A12=1,A12="да",A12="ДА",A12="ИСТИНА"),ROUND(C12*D12*E12/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K12">
-        <f>IF(A12&lt;&gt;TRUE,"",ROUND((N(F12)*C12+N(G12)*C12+N(H12)*D12+N(I12)*D12)*E12/1000,3))</f>
+        <f>IF(OR(A12=1,A12="да",A12="ДА",A12="ИСТИНА"),ROUND((IF(OR(F12=1,F12="да",F12="ДА",F12="ИСТИНА"),C12,0)+IF(OR(G12=1,G12="да",G12="ДА",G12="ИСТИНА"),C12,0)+IF(OR(H12=1,H12="да",H12="ДА",H12="ИСТИНА"),D12,0)+IF(OR(I12=1,I12="да",I12="ДА",I12="ИСТИНА"),D12,0))*E12/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L12">
-        <f>IF(A12&lt;&gt;TRUE,"",ROUND((C12+D12)*2*E12/1000,3))</f>
+        <f>IF(OR(A12=1,A12="да",A12="ДА",A12="ИСТИНА"),ROUND((C12+D12)*2*E12/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="b">
+      <c r="A13">
         <v>0</v>
       </c>
       <c r="B13" t="str">
@@ -1742,33 +1742,33 @@
       <c r="E13" t="str">
         <v/>
       </c>
-      <c r="F13" t="b">
-        <v>0</v>
-      </c>
-      <c r="G13" t="b">
-        <v>0</v>
-      </c>
-      <c r="H13" t="b">
-        <v>0</v>
-      </c>
-      <c r="I13" t="b">
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
         <v>0</v>
       </c>
       <c r="J13">
-        <f>IF(A13&lt;&gt;TRUE,"",ROUND(C13*D13*E13/1000000,3))</f>
+        <f>IF(OR(A13=1,A13="да",A13="ДА",A13="ИСТИНА"),ROUND(C13*D13*E13/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K13">
-        <f>IF(A13&lt;&gt;TRUE,"",ROUND((N(F13)*C13+N(G13)*C13+N(H13)*D13+N(I13)*D13)*E13/1000,3))</f>
+        <f>IF(OR(A13=1,A13="да",A13="ДА",A13="ИСТИНА"),ROUND((IF(OR(F13=1,F13="да",F13="ДА",F13="ИСТИНА"),C13,0)+IF(OR(G13=1,G13="да",G13="ДА",G13="ИСТИНА"),C13,0)+IF(OR(H13=1,H13="да",H13="ДА",H13="ИСТИНА"),D13,0)+IF(OR(I13=1,I13="да",I13="ДА",I13="ИСТИНА"),D13,0))*E13/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L13">
-        <f>IF(A13&lt;&gt;TRUE,"",ROUND((C13+D13)*2*E13/1000,3))</f>
+        <f>IF(OR(A13=1,A13="да",A13="ДА",A13="ИСТИНА"),ROUND((C13+D13)*2*E13/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="b">
+      <c r="A14">
         <v>0</v>
       </c>
       <c r="B14" t="str">
@@ -1783,33 +1783,33 @@
       <c r="E14" t="str">
         <v/>
       </c>
-      <c r="F14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" t="b">
-        <v>0</v>
-      </c>
-      <c r="H14" t="b">
-        <v>0</v>
-      </c>
-      <c r="I14" t="b">
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
         <v>0</v>
       </c>
       <c r="J14">
-        <f>IF(A14&lt;&gt;TRUE,"",ROUND(C14*D14*E14/1000000,3))</f>
+        <f>IF(OR(A14=1,A14="да",A14="ДА",A14="ИСТИНА"),ROUND(C14*D14*E14/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K14">
-        <f>IF(A14&lt;&gt;TRUE,"",ROUND((N(F14)*C14+N(G14)*C14+N(H14)*D14+N(I14)*D14)*E14/1000,3))</f>
+        <f>IF(OR(A14=1,A14="да",A14="ДА",A14="ИСТИНА"),ROUND((IF(OR(F14=1,F14="да",F14="ДА",F14="ИСТИНА"),C14,0)+IF(OR(G14=1,G14="да",G14="ДА",G14="ИСТИНА"),C14,0)+IF(OR(H14=1,H14="да",H14="ДА",H14="ИСТИНА"),D14,0)+IF(OR(I14=1,I14="да",I14="ДА",I14="ИСТИНА"),D14,0))*E14/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L14">
-        <f>IF(A14&lt;&gt;TRUE,"",ROUND((C14+D14)*2*E14/1000,3))</f>
+        <f>IF(OR(A14=1,A14="да",A14="ДА",A14="ИСТИНА"),ROUND((C14+D14)*2*E14/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="b">
+      <c r="A15">
         <v>0</v>
       </c>
       <c r="B15" t="str">
@@ -1824,28 +1824,28 @@
       <c r="E15" t="str">
         <v/>
       </c>
-      <c r="F15" t="b">
-        <v>0</v>
-      </c>
-      <c r="G15" t="b">
-        <v>0</v>
-      </c>
-      <c r="H15" t="b">
-        <v>0</v>
-      </c>
-      <c r="I15" t="b">
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
         <v>0</v>
       </c>
       <c r="J15">
-        <f>IF(A15&lt;&gt;TRUE,"",ROUND(C15*D15*E15/1000000,3))</f>
+        <f>IF(OR(A15=1,A15="да",A15="ДА",A15="ИСТИНА"),ROUND(C15*D15*E15/1000000,3),"")</f>
         <v>0</v>
       </c>
       <c r="K15">
-        <f>IF(A15&lt;&gt;TRUE,"",ROUND((N(F15)*C15+N(G15)*C15+N(H15)*D15+N(I15)*D15)*E15/1000,3))</f>
+        <f>IF(OR(A15=1,A15="да",A15="ДА",A15="ИСТИНА"),ROUND((IF(OR(F15=1,F15="да",F15="ДА",F15="ИСТИНА"),C15,0)+IF(OR(G15=1,G15="да",G15="ДА",G15="ИСТИНА"),C15,0)+IF(OR(H15=1,H15="да",H15="ДА",H15="ИСТИНА"),D15,0)+IF(OR(I15=1,I15="да",I15="ДА",I15="ИСТИНА"),D15,0))*E15/1000,3),"")</f>
         <v>0</v>
       </c>
       <c r="L15">
-        <f>IF(A15&lt;&gt;TRUE,"",ROUND((C15+D15)*2*E15/1000,3))</f>
+        <f>IF(OR(A15=1,A15="да",A15="ДА",A15="ИСТИНА"),ROUND((C15+D15)*2*E15/1000,3),"")</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>